<commit_message>
Word export (all 3 tools): fix missing styles.xml causing every paragraph/blank line to inherit Word's own ~8pt default spacing when opened or copied from the exported doc — explicit zero-spacing Normal style + zero-spacing blank-line paragraphs; medication chart template: bigger date/AM-PM rows and font, still fits one printed page (width was the binding constraint, not height); Surgery: oral meloxicam AM/PM default now driven by Surgery end time for both cats and dogs (was: dog-only, tied to the Meloxicam SC tick time; cats had a manual picker)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/template/medication-chart-template.xlsx
+++ b/template/medication-chart-template.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="dd-mmm"/>
     <numFmt numFmtId="165" formatCode="0.##"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -70,6 +70,10 @@
     <font>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -353,7 +357,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -467,6 +471,12 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1359,7 +1369,7 @@
       </c>
       <c r="S15" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve">D</t>
+          <t>D</t>
         </is>
       </c>
       <c r="T15" s="59" t="inlineStr">
@@ -1378,12 +1388,12 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="12" customHeight="1">
-      <c r="A16" s="27">
+    <row r="16" ht="17" customHeight="1">
+      <c r="A16" s="62">
         <f>TODAY()+1</f>
         <v/>
       </c>
-      <c r="B16" s="28" t="inlineStr">
+      <c r="B16" s="63" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -1429,7 +1439,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="12" customHeight="1">
+    <row r="17" ht="17" customHeight="1">
       <c r="A17" s="54" t="n"/>
       <c r="B17" s="54" t="n"/>
       <c r="C17" s="34" t="n"/>
@@ -1472,12 +1482,12 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="12" customHeight="1">
-      <c r="A18" s="27">
+    <row r="18" ht="17" customHeight="1">
+      <c r="A18" s="62">
         <f>A16+1</f>
         <v/>
       </c>
-      <c r="B18" s="28" t="inlineStr">
+      <c r="B18" s="63" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -1523,7 +1533,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="12" customHeight="1">
+    <row r="19" ht="17" customHeight="1">
       <c r="A19" s="54" t="n"/>
       <c r="B19" s="54" t="n"/>
       <c r="C19" s="34" t="n"/>
@@ -1566,12 +1576,12 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="12" customHeight="1">
-      <c r="A20" s="27">
+    <row r="20" ht="17" customHeight="1">
+      <c r="A20" s="62">
         <f>A18+1</f>
         <v/>
       </c>
-      <c r="B20" s="28" t="inlineStr">
+      <c r="B20" s="63" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -1617,7 +1627,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="12" customHeight="1">
+    <row r="21" ht="17" customHeight="1">
       <c r="A21" s="54" t="n"/>
       <c r="B21" s="54" t="n"/>
       <c r="C21" s="34" t="n"/>
@@ -1660,12 +1670,12 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="12" customHeight="1">
-      <c r="A22" s="27">
+    <row r="22" ht="17" customHeight="1">
+      <c r="A22" s="62">
         <f>A20+1</f>
         <v/>
       </c>
-      <c r="B22" s="28" t="inlineStr">
+      <c r="B22" s="63" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -1711,7 +1721,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="12" customHeight="1">
+    <row r="23" ht="17" customHeight="1">
       <c r="A23" s="54" t="n"/>
       <c r="B23" s="54" t="n"/>
       <c r="C23" s="34" t="n"/>
@@ -1754,12 +1764,12 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="12" customHeight="1">
-      <c r="A24" s="27">
+    <row r="24" ht="17" customHeight="1">
+      <c r="A24" s="62">
         <f>A22+1</f>
         <v/>
       </c>
-      <c r="B24" s="28" t="inlineStr">
+      <c r="B24" s="63" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -1800,7 +1810,7 @@
       <c r="T24" s="60" t="n"/>
       <c r="U24" s="60" t="n"/>
     </row>
-    <row r="25" ht="12" customHeight="1">
+    <row r="25" ht="17" customHeight="1">
       <c r="A25" s="54" t="n"/>
       <c r="B25" s="54" t="n"/>
       <c r="C25" s="34" t="n"/>
@@ -1838,12 +1848,12 @@
       <c r="T25" s="54" t="n"/>
       <c r="U25" s="54" t="n"/>
     </row>
-    <row r="26" ht="12" customHeight="1">
-      <c r="A26" s="27">
+    <row r="26" ht="17" customHeight="1">
+      <c r="A26" s="62">
         <f>A24+1</f>
         <v/>
       </c>
-      <c r="B26" s="28" t="inlineStr">
+      <c r="B26" s="63" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -1884,7 +1894,7 @@
       <c r="T26" s="60" t="n"/>
       <c r="U26" s="60" t="n"/>
     </row>
-    <row r="27" ht="12" customHeight="1">
+    <row r="27" ht="17" customHeight="1">
       <c r="A27" s="54" t="n"/>
       <c r="B27" s="54" t="n"/>
       <c r="C27" s="34" t="n"/>
@@ -1922,12 +1932,12 @@
       <c r="T27" s="54" t="n"/>
       <c r="U27" s="54" t="n"/>
     </row>
-    <row r="28" ht="12" customHeight="1">
-      <c r="A28" s="27">
+    <row r="28" ht="17" customHeight="1">
+      <c r="A28" s="62">
         <f>A26+1</f>
         <v/>
       </c>
-      <c r="B28" s="28" t="inlineStr">
+      <c r="B28" s="63" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -1968,7 +1978,7 @@
       <c r="T28" s="60" t="n"/>
       <c r="U28" s="60" t="n"/>
     </row>
-    <row r="29" ht="12" customHeight="1">
+    <row r="29" ht="17" customHeight="1">
       <c r="A29" s="54" t="n"/>
       <c r="B29" s="54" t="n"/>
       <c r="C29" s="34" t="n"/>
@@ -2006,12 +2016,12 @@
       <c r="T29" s="54" t="n"/>
       <c r="U29" s="54" t="n"/>
     </row>
-    <row r="30" ht="12" customHeight="1">
-      <c r="A30" s="27">
+    <row r="30" ht="17" customHeight="1">
+      <c r="A30" s="62">
         <f>A28+1</f>
         <v/>
       </c>
-      <c r="B30" s="28" t="inlineStr">
+      <c r="B30" s="63" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -2052,7 +2062,7 @@
       <c r="T30" s="60" t="n"/>
       <c r="U30" s="60" t="n"/>
     </row>
-    <row r="31" ht="12" customHeight="1">
+    <row r="31" ht="17" customHeight="1">
       <c r="A31" s="54" t="n"/>
       <c r="B31" s="54" t="n"/>
       <c r="C31" s="34" t="n"/>
@@ -2090,12 +2100,12 @@
       <c r="T31" s="54" t="n"/>
       <c r="U31" s="54" t="n"/>
     </row>
-    <row r="32" ht="12" customHeight="1">
-      <c r="A32" s="27">
+    <row r="32" ht="17" customHeight="1">
+      <c r="A32" s="62">
         <f>A30+1</f>
         <v/>
       </c>
-      <c r="B32" s="28" t="inlineStr">
+      <c r="B32" s="63" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -2136,7 +2146,7 @@
       <c r="T32" s="60" t="n"/>
       <c r="U32" s="60" t="n"/>
     </row>
-    <row r="33" ht="12" customHeight="1">
+    <row r="33" ht="17" customHeight="1">
       <c r="A33" s="54" t="n"/>
       <c r="B33" s="54" t="n"/>
       <c r="C33" s="34" t="n"/>
@@ -2174,12 +2184,12 @@
       <c r="T33" s="54" t="n"/>
       <c r="U33" s="54" t="n"/>
     </row>
-    <row r="34" ht="12" customHeight="1">
-      <c r="A34" s="27">
+    <row r="34" ht="17" customHeight="1">
+      <c r="A34" s="62">
         <f>A32+1</f>
         <v/>
       </c>
-      <c r="B34" s="28" t="inlineStr">
+      <c r="B34" s="63" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -2220,7 +2230,7 @@
       <c r="T34" s="60" t="n"/>
       <c r="U34" s="60" t="n"/>
     </row>
-    <row r="35" ht="12" customHeight="1">
+    <row r="35" ht="17" customHeight="1">
       <c r="A35" s="54" t="n"/>
       <c r="B35" s="54" t="n"/>
       <c r="C35" s="34" t="n"/>
@@ -2258,12 +2268,12 @@
       <c r="T35" s="54" t="n"/>
       <c r="U35" s="54" t="n"/>
     </row>
-    <row r="36" ht="12" customHeight="1">
-      <c r="A36" s="27">
+    <row r="36" ht="17" customHeight="1">
+      <c r="A36" s="62">
         <f>A34+1</f>
         <v/>
       </c>
-      <c r="B36" s="28" t="inlineStr">
+      <c r="B36" s="63" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -2304,7 +2314,7 @@
       <c r="T36" s="60" t="n"/>
       <c r="U36" s="60" t="n"/>
     </row>
-    <row r="37" ht="12" customHeight="1">
+    <row r="37" ht="17" customHeight="1">
       <c r="A37" s="54" t="n"/>
       <c r="B37" s="54" t="n"/>
       <c r="C37" s="34" t="n"/>
@@ -2342,12 +2352,12 @@
       <c r="T37" s="54" t="n"/>
       <c r="U37" s="54" t="n"/>
     </row>
-    <row r="38" ht="12" customHeight="1">
-      <c r="A38" s="27">
+    <row r="38" ht="17" customHeight="1">
+      <c r="A38" s="62">
         <f>A36+1</f>
         <v/>
       </c>
-      <c r="B38" s="28" t="inlineStr">
+      <c r="B38" s="63" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -2388,7 +2398,7 @@
       <c r="T38" s="60" t="n"/>
       <c r="U38" s="60" t="n"/>
     </row>
-    <row r="39" ht="12" customHeight="1">
+    <row r="39" ht="17" customHeight="1">
       <c r="A39" s="54" t="n"/>
       <c r="B39" s="54" t="n"/>
       <c r="C39" s="34" t="n"/>
@@ -2426,12 +2436,12 @@
       <c r="T39" s="54" t="n"/>
       <c r="U39" s="54" t="n"/>
     </row>
-    <row r="40" ht="12" customHeight="1">
-      <c r="A40" s="27">
+    <row r="40" ht="17" customHeight="1">
+      <c r="A40" s="62">
         <f>A38+1</f>
         <v/>
       </c>
-      <c r="B40" s="28" t="inlineStr">
+      <c r="B40" s="63" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -2472,7 +2482,7 @@
       <c r="T40" s="60" t="n"/>
       <c r="U40" s="60" t="n"/>
     </row>
-    <row r="41" ht="12" customHeight="1">
+    <row r="41" ht="17" customHeight="1">
       <c r="A41" s="54" t="n"/>
       <c r="B41" s="54" t="n"/>
       <c r="C41" s="34" t="n"/>
@@ -2510,12 +2520,12 @@
       <c r="T41" s="54" t="n"/>
       <c r="U41" s="54" t="n"/>
     </row>
-    <row r="42" ht="12" customHeight="1">
-      <c r="A42" s="27">
+    <row r="42" ht="17" customHeight="1">
+      <c r="A42" s="62">
         <f>A40+1</f>
         <v/>
       </c>
-      <c r="B42" s="28" t="inlineStr">
+      <c r="B42" s="63" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -2556,7 +2566,7 @@
       <c r="T42" s="60" t="n"/>
       <c r="U42" s="60" t="n"/>
     </row>
-    <row r="43" ht="12" customHeight="1">
+    <row r="43" ht="17" customHeight="1">
       <c r="A43" s="54" t="n"/>
       <c r="B43" s="54" t="n"/>
       <c r="C43" s="37" t="n"/>

</xml_diff>

<commit_message>
Medication chart template: remove Date Dispensed/Quantity/legend section, make the 14-day grid bigger again with the freed space (20pt rows, larger date/AM-PM font), freeze panes on the header block so Patient ID stays visible while scrolling the grid; medication-charts.html print-area range updated to match the shorter sheet
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/template/medication-chart-template.xlsx
+++ b/template/medication-chart-template.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Sheet1'!$A$1:$U$48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Sheet1'!$A$1:$U$43</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="dd-mmm"/>
     <numFmt numFmtId="165" formatCode="0.##"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,6 +74,10 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -357,7 +361,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -476,6 +480,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -860,7 +870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Y48"/>
+  <dimension ref="A1:Y43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.5" customWidth="1" min="1" max="1"/>
@@ -1388,12 +1398,12 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="17" customHeight="1">
-      <c r="A16" s="62">
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="64">
         <f>TODAY()+1</f>
         <v/>
       </c>
-      <c r="B16" s="63" t="inlineStr">
+      <c r="B16" s="65" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -1439,7 +1449,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="17" customHeight="1">
+    <row r="17" ht="20" customHeight="1">
       <c r="A17" s="54" t="n"/>
       <c r="B17" s="54" t="n"/>
       <c r="C17" s="34" t="n"/>
@@ -1482,12 +1492,12 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="17" customHeight="1">
-      <c r="A18" s="62">
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="64">
         <f>A16+1</f>
         <v/>
       </c>
-      <c r="B18" s="63" t="inlineStr">
+      <c r="B18" s="65" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -1533,7 +1543,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="17" customHeight="1">
+    <row r="19" ht="20" customHeight="1">
       <c r="A19" s="54" t="n"/>
       <c r="B19" s="54" t="n"/>
       <c r="C19" s="34" t="n"/>
@@ -1576,12 +1586,12 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="17" customHeight="1">
-      <c r="A20" s="62">
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="64">
         <f>A18+1</f>
         <v/>
       </c>
-      <c r="B20" s="63" t="inlineStr">
+      <c r="B20" s="65" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -1627,7 +1637,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="17" customHeight="1">
+    <row r="21" ht="20" customHeight="1">
       <c r="A21" s="54" t="n"/>
       <c r="B21" s="54" t="n"/>
       <c r="C21" s="34" t="n"/>
@@ -1670,12 +1680,12 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="17" customHeight="1">
-      <c r="A22" s="62">
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="64">
         <f>A20+1</f>
         <v/>
       </c>
-      <c r="B22" s="63" t="inlineStr">
+      <c r="B22" s="65" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -1721,7 +1731,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="17" customHeight="1">
+    <row r="23" ht="20" customHeight="1">
       <c r="A23" s="54" t="n"/>
       <c r="B23" s="54" t="n"/>
       <c r="C23" s="34" t="n"/>
@@ -1764,12 +1774,12 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="17" customHeight="1">
-      <c r="A24" s="62">
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="64">
         <f>A22+1</f>
         <v/>
       </c>
-      <c r="B24" s="63" t="inlineStr">
+      <c r="B24" s="65" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -1810,7 +1820,7 @@
       <c r="T24" s="60" t="n"/>
       <c r="U24" s="60" t="n"/>
     </row>
-    <row r="25" ht="17" customHeight="1">
+    <row r="25" ht="20" customHeight="1">
       <c r="A25" s="54" t="n"/>
       <c r="B25" s="54" t="n"/>
       <c r="C25" s="34" t="n"/>
@@ -1848,12 +1858,12 @@
       <c r="T25" s="54" t="n"/>
       <c r="U25" s="54" t="n"/>
     </row>
-    <row r="26" ht="17" customHeight="1">
-      <c r="A26" s="62">
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="64">
         <f>A24+1</f>
         <v/>
       </c>
-      <c r="B26" s="63" t="inlineStr">
+      <c r="B26" s="65" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -1894,7 +1904,7 @@
       <c r="T26" s="60" t="n"/>
       <c r="U26" s="60" t="n"/>
     </row>
-    <row r="27" ht="17" customHeight="1">
+    <row r="27" ht="20" customHeight="1">
       <c r="A27" s="54" t="n"/>
       <c r="B27" s="54" t="n"/>
       <c r="C27" s="34" t="n"/>
@@ -1932,12 +1942,12 @@
       <c r="T27" s="54" t="n"/>
       <c r="U27" s="54" t="n"/>
     </row>
-    <row r="28" ht="17" customHeight="1">
-      <c r="A28" s="62">
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="64">
         <f>A26+1</f>
         <v/>
       </c>
-      <c r="B28" s="63" t="inlineStr">
+      <c r="B28" s="65" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -1978,7 +1988,7 @@
       <c r="T28" s="60" t="n"/>
       <c r="U28" s="60" t="n"/>
     </row>
-    <row r="29" ht="17" customHeight="1">
+    <row r="29" ht="20" customHeight="1">
       <c r="A29" s="54" t="n"/>
       <c r="B29" s="54" t="n"/>
       <c r="C29" s="34" t="n"/>
@@ -2016,12 +2026,12 @@
       <c r="T29" s="54" t="n"/>
       <c r="U29" s="54" t="n"/>
     </row>
-    <row r="30" ht="17" customHeight="1">
-      <c r="A30" s="62">
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="64">
         <f>A28+1</f>
         <v/>
       </c>
-      <c r="B30" s="63" t="inlineStr">
+      <c r="B30" s="65" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -2062,7 +2072,7 @@
       <c r="T30" s="60" t="n"/>
       <c r="U30" s="60" t="n"/>
     </row>
-    <row r="31" ht="17" customHeight="1">
+    <row r="31" ht="20" customHeight="1">
       <c r="A31" s="54" t="n"/>
       <c r="B31" s="54" t="n"/>
       <c r="C31" s="34" t="n"/>
@@ -2100,12 +2110,12 @@
       <c r="T31" s="54" t="n"/>
       <c r="U31" s="54" t="n"/>
     </row>
-    <row r="32" ht="17" customHeight="1">
-      <c r="A32" s="62">
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="64">
         <f>A30+1</f>
         <v/>
       </c>
-      <c r="B32" s="63" t="inlineStr">
+      <c r="B32" s="65" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -2146,7 +2156,7 @@
       <c r="T32" s="60" t="n"/>
       <c r="U32" s="60" t="n"/>
     </row>
-    <row r="33" ht="17" customHeight="1">
+    <row r="33" ht="20" customHeight="1">
       <c r="A33" s="54" t="n"/>
       <c r="B33" s="54" t="n"/>
       <c r="C33" s="34" t="n"/>
@@ -2184,12 +2194,12 @@
       <c r="T33" s="54" t="n"/>
       <c r="U33" s="54" t="n"/>
     </row>
-    <row r="34" ht="17" customHeight="1">
-      <c r="A34" s="62">
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="64">
         <f>A32+1</f>
         <v/>
       </c>
-      <c r="B34" s="63" t="inlineStr">
+      <c r="B34" s="65" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -2230,7 +2240,7 @@
       <c r="T34" s="60" t="n"/>
       <c r="U34" s="60" t="n"/>
     </row>
-    <row r="35" ht="17" customHeight="1">
+    <row r="35" ht="20" customHeight="1">
       <c r="A35" s="54" t="n"/>
       <c r="B35" s="54" t="n"/>
       <c r="C35" s="34" t="n"/>
@@ -2268,12 +2278,12 @@
       <c r="T35" s="54" t="n"/>
       <c r="U35" s="54" t="n"/>
     </row>
-    <row r="36" ht="17" customHeight="1">
-      <c r="A36" s="62">
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="64">
         <f>A34+1</f>
         <v/>
       </c>
-      <c r="B36" s="63" t="inlineStr">
+      <c r="B36" s="65" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -2314,7 +2324,7 @@
       <c r="T36" s="60" t="n"/>
       <c r="U36" s="60" t="n"/>
     </row>
-    <row r="37" ht="17" customHeight="1">
+    <row r="37" ht="20" customHeight="1">
       <c r="A37" s="54" t="n"/>
       <c r="B37" s="54" t="n"/>
       <c r="C37" s="34" t="n"/>
@@ -2352,12 +2362,12 @@
       <c r="T37" s="54" t="n"/>
       <c r="U37" s="54" t="n"/>
     </row>
-    <row r="38" ht="17" customHeight="1">
-      <c r="A38" s="62">
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="64">
         <f>A36+1</f>
         <v/>
       </c>
-      <c r="B38" s="63" t="inlineStr">
+      <c r="B38" s="65" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -2398,7 +2408,7 @@
       <c r="T38" s="60" t="n"/>
       <c r="U38" s="60" t="n"/>
     </row>
-    <row r="39" ht="17" customHeight="1">
+    <row r="39" ht="20" customHeight="1">
       <c r="A39" s="54" t="n"/>
       <c r="B39" s="54" t="n"/>
       <c r="C39" s="34" t="n"/>
@@ -2436,12 +2446,12 @@
       <c r="T39" s="54" t="n"/>
       <c r="U39" s="54" t="n"/>
     </row>
-    <row r="40" ht="17" customHeight="1">
-      <c r="A40" s="62">
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="64">
         <f>A38+1</f>
         <v/>
       </c>
-      <c r="B40" s="63" t="inlineStr">
+      <c r="B40" s="65" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -2482,7 +2492,7 @@
       <c r="T40" s="60" t="n"/>
       <c r="U40" s="60" t="n"/>
     </row>
-    <row r="41" ht="17" customHeight="1">
+    <row r="41" ht="20" customHeight="1">
       <c r="A41" s="54" t="n"/>
       <c r="B41" s="54" t="n"/>
       <c r="C41" s="34" t="n"/>
@@ -2520,12 +2530,12 @@
       <c r="T41" s="54" t="n"/>
       <c r="U41" s="54" t="n"/>
     </row>
-    <row r="42" ht="17" customHeight="1">
-      <c r="A42" s="62">
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="64">
         <f>A40+1</f>
         <v/>
       </c>
-      <c r="B42" s="63" t="inlineStr">
+      <c r="B42" s="65" t="inlineStr">
         <is>
           <t>AM
 PM</t>
@@ -2566,7 +2576,7 @@
       <c r="T42" s="60" t="n"/>
       <c r="U42" s="60" t="n"/>
     </row>
-    <row r="43" ht="17" customHeight="1">
+    <row r="43" ht="20" customHeight="1">
       <c r="A43" s="54" t="n"/>
       <c r="B43" s="54" t="n"/>
       <c r="C43" s="37" t="n"/>
@@ -2605,29 +2615,10 @@
       <c r="U43" s="54" t="n"/>
     </row>
     <row r="44" ht="4" customHeight="1"/>
-    <row r="45" ht="12" customHeight="1">
-      <c r="A45" s="41" t="inlineStr">
-        <is>
-          <t>Date Dispensed</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="12" customHeight="1">
-      <c r="A46" s="42" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-    </row>
+    <row r="45" ht="12" customHeight="1"/>
+    <row r="46" ht="12" customHeight="1"/>
     <row r="47" ht="4" customHeight="1"/>
-    <row r="48" ht="12" customHeight="1">
-      <c r="A48" s="61" t="inlineStr">
-        <is>
-          <t>R/C = Recheck with vet before continuing / stopping medication.
-E = Eating, D = Drinking, U = Urinating, D = Defecating — score 0-3 each visit.</t>
-        </is>
-      </c>
-    </row>
+    <row r="48" ht="12" customHeight="1"/>
   </sheetData>
   <mergeCells count="132">
     <mergeCell ref="F8:H8"/>

</xml_diff>

<commit_message>
Medication chart template: bigger fonts for Patient ID, medication label, dose, freq, route and days; removed the freeze pane (not needed for this sheet after all)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/template/medication-chart-template.xlsx
+++ b/template/medication-chart-template.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="dd-mmm"/>
     <numFmt numFmtId="165" formatCode="0.##"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -78,6 +78,9 @@
       <b val="1"/>
       <sz val="13"/>
     </font>
+    <font>
+      <sz val="13"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -361,7 +364,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -487,6 +490,21 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -926,7 +944,7 @@
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="66" t="inlineStr">
         <is>
           <t>Patient ID:</t>
         </is>
@@ -1139,19 +1157,19 @@
       </c>
     </row>
     <row r="9" ht="13" customHeight="1">
-      <c r="C9" s="10" t="inlineStr"/>
+      <c r="C9" s="67" t="inlineStr"/>
       <c r="D9" s="11" t="n"/>
       <c r="E9" s="12" t="n"/>
-      <c r="F9" s="10" t="inlineStr"/>
+      <c r="F9" s="67" t="inlineStr"/>
       <c r="G9" s="11" t="n"/>
       <c r="H9" s="12" t="n"/>
-      <c r="I9" s="10" t="inlineStr"/>
+      <c r="I9" s="67" t="inlineStr"/>
       <c r="J9" s="11" t="n"/>
       <c r="K9" s="12" t="n"/>
-      <c r="L9" s="10" t="inlineStr"/>
+      <c r="L9" s="67" t="inlineStr"/>
       <c r="M9" s="11" t="n"/>
       <c r="N9" s="12" t="n"/>
-      <c r="O9" s="10" t="inlineStr"/>
+      <c r="O9" s="67" t="inlineStr"/>
       <c r="P9" s="11" t="n"/>
       <c r="Q9" s="12" t="n"/>
       <c r="Y9" t="inlineStr">
@@ -1166,35 +1184,35 @@
           <t>Days:</t>
         </is>
       </c>
-      <c r="D10" s="14" t="n"/>
+      <c r="D10" s="68" t="n"/>
       <c r="E10" s="15" t="n"/>
       <c r="F10" s="13" t="inlineStr">
         <is>
           <t>Days:</t>
         </is>
       </c>
-      <c r="G10" s="14" t="n"/>
+      <c r="G10" s="68" t="n"/>
       <c r="H10" s="15" t="n"/>
       <c r="I10" s="13" t="inlineStr">
         <is>
           <t>Days:</t>
         </is>
       </c>
-      <c r="J10" s="14" t="n"/>
+      <c r="J10" s="68" t="n"/>
       <c r="K10" s="15" t="n"/>
       <c r="L10" s="13" t="inlineStr">
         <is>
           <t>Days:</t>
         </is>
       </c>
-      <c r="M10" s="14" t="n"/>
+      <c r="M10" s="68" t="n"/>
       <c r="N10" s="15" t="n"/>
       <c r="O10" s="13" t="inlineStr">
         <is>
           <t>Days:</t>
         </is>
       </c>
-      <c r="P10" s="14" t="n"/>
+      <c r="P10" s="68" t="n"/>
       <c r="Q10" s="15" t="n"/>
       <c r="Y10" t="inlineStr">
         <is>
@@ -1240,31 +1258,31 @@
       </c>
     </row>
     <row r="12" ht="14" customHeight="1">
-      <c r="C12" s="17">
+      <c r="C12" s="69">
         <f>"Dose: "&amp;IF(OR($B$8="",NOT(ISNUMBER($B$8))),"",IF(C9="Amoxyclav 50mg",CEILING($B$8*20/50,0.25)&amp;" tablets",IF(C9="Amoxyclav 250mg",CEILING($B$8*20/250,0.25)&amp;" tablets",IF(C9="Amoxyclav 500mg",CEILING($B$8*20/500,0.25)&amp;" tablets",IF(C9="Doxycycline 50mg",CEILING($B$8*10/50,0.25)&amp;" tablets",IF(C9="Doxycycline 100mg",CEILING($B$8*10/100,0.25)&amp;" tablets",IF(C9="Famvir 125mg",CEILING($B$8*90/125,0.25)&amp;" tablets",IF(C9="Famvir 250mg",CEILING($B$8*90/250,0.25)&amp;" tablets",IF(C9="Meloxicam 1mg (dog tablet)",CEILING($B$8*0.1/1,0.25)&amp;" tablets",IF(C9="Meloxicam 2.5mg (dog tablet)",CEILING($B$8*0.1/2.5,0.25)&amp;" tablets",IF(C9="Clavulox drops (62.5mg/mL)",ROUND($B$8*20/62.5,2)&amp;"mL",IF(C9="Paracetamol 500mg (DOGS ONLY)",CEILING($B$8*15/500,0.25)&amp;" tablets",IF(C9="Doxybrom",ROUND($B$8*0.05,2)&amp;"mL",IF(C9="Panacur",ROUND($B$8/2,2)&amp;"mL",IF(C9="Famvir 250mg/mL solution",ROUND($B$8*90/250,2)&amp;"mL",IF(C9="Mirtazapine 1.88mg (transdermal)","1.88mg",IF(C9="Buprenorphine",ROUND($B$8*0.02/0.3,2)&amp;"mL",IF(C9="Doxycycline paste",CEILING($B$8*10/25,0.5)&amp;" notches",IF(C9="Meloxicam (cat, liquid)",ROUND($B$8*0.1,2)&amp;"mL",IF(C9="Meloxicam (dog, liquid)",ROUND($B$8*0.1/5,2)&amp;"mL",""))))))))))))))))))))</f>
         <v/>
       </c>
       <c r="D12" s="11" t="n"/>
       <c r="E12" s="12" t="n"/>
-      <c r="F12" s="17">
+      <c r="F12" s="69">
         <f>"Dose: "&amp;IF(OR($B$8="",NOT(ISNUMBER($B$8))),"",IF(F9="Amoxyclav 50mg",CEILING($B$8*20/50,0.25)&amp;" tablets",IF(F9="Amoxyclav 250mg",CEILING($B$8*20/250,0.25)&amp;" tablets",IF(F9="Amoxyclav 500mg",CEILING($B$8*20/500,0.25)&amp;" tablets",IF(F9="Doxycycline 50mg",CEILING($B$8*10/50,0.25)&amp;" tablets",IF(F9="Doxycycline 100mg",CEILING($B$8*10/100,0.25)&amp;" tablets",IF(F9="Famvir 125mg",CEILING($B$8*90/125,0.25)&amp;" tablets",IF(F9="Famvir 250mg",CEILING($B$8*90/250,0.25)&amp;" tablets",IF(F9="Meloxicam 1mg (dog tablet)",CEILING($B$8*0.1/1,0.25)&amp;" tablets",IF(F9="Meloxicam 2.5mg (dog tablet)",CEILING($B$8*0.1/2.5,0.25)&amp;" tablets",IF(F9="Clavulox drops (62.5mg/mL)",ROUND($B$8*20/62.5,2)&amp;"mL",IF(F9="Paracetamol 500mg (DOGS ONLY)",CEILING($B$8*15/500,0.25)&amp;" tablets",IF(F9="Doxybrom",ROUND($B$8*0.05,2)&amp;"mL",IF(F9="Panacur",ROUND($B$8/2,2)&amp;"mL",IF(F9="Famvir 250mg/mL solution",ROUND($B$8*90/250,2)&amp;"mL",IF(F9="Mirtazapine 1.88mg (transdermal)","1.88mg",IF(F9="Buprenorphine",ROUND($B$8*0.02/0.3,2)&amp;"mL",IF(F9="Doxycycline paste",CEILING($B$8*10/25,0.5)&amp;" notches",IF(F9="Meloxicam (cat, liquid)",ROUND($B$8*0.1,2)&amp;"mL",IF(F9="Meloxicam (dog, liquid)",ROUND($B$8*0.1/5,2)&amp;"mL",""))))))))))))))))))))</f>
         <v/>
       </c>
       <c r="G12" s="11" t="n"/>
       <c r="H12" s="12" t="n"/>
-      <c r="I12" s="17">
+      <c r="I12" s="69">
         <f>"Dose: "&amp;IF(OR($B$8="",NOT(ISNUMBER($B$8))),"",IF(I9="Amoxyclav 50mg",CEILING($B$8*20/50,0.25)&amp;" tablets",IF(I9="Amoxyclav 250mg",CEILING($B$8*20/250,0.25)&amp;" tablets",IF(I9="Amoxyclav 500mg",CEILING($B$8*20/500,0.25)&amp;" tablets",IF(I9="Doxycycline 50mg",CEILING($B$8*10/50,0.25)&amp;" tablets",IF(I9="Doxycycline 100mg",CEILING($B$8*10/100,0.25)&amp;" tablets",IF(I9="Famvir 125mg",CEILING($B$8*90/125,0.25)&amp;" tablets",IF(I9="Famvir 250mg",CEILING($B$8*90/250,0.25)&amp;" tablets",IF(I9="Meloxicam 1mg (dog tablet)",CEILING($B$8*0.1/1,0.25)&amp;" tablets",IF(I9="Meloxicam 2.5mg (dog tablet)",CEILING($B$8*0.1/2.5,0.25)&amp;" tablets",IF(I9="Clavulox drops (62.5mg/mL)",ROUND($B$8*20/62.5,2)&amp;"mL",IF(I9="Paracetamol 500mg (DOGS ONLY)",CEILING($B$8*15/500,0.25)&amp;" tablets",IF(I9="Doxybrom",ROUND($B$8*0.05,2)&amp;"mL",IF(I9="Panacur",ROUND($B$8/2,2)&amp;"mL",IF(I9="Famvir 250mg/mL solution",ROUND($B$8*90/250,2)&amp;"mL",IF(I9="Mirtazapine 1.88mg (transdermal)","1.88mg",IF(I9="Buprenorphine",ROUND($B$8*0.02/0.3,2)&amp;"mL",IF(I9="Doxycycline paste",CEILING($B$8*10/25,0.5)&amp;" notches",IF(I9="Meloxicam (cat, liquid)",ROUND($B$8*0.1,2)&amp;"mL",IF(I9="Meloxicam (dog, liquid)",ROUND($B$8*0.1/5,2)&amp;"mL",""))))))))))))))))))))</f>
         <v/>
       </c>
       <c r="J12" s="11" t="n"/>
       <c r="K12" s="12" t="n"/>
-      <c r="L12" s="17">
+      <c r="L12" s="69">
         <f>"Dose: "&amp;IF(OR($B$8="",NOT(ISNUMBER($B$8))),"",IF(L9="Amoxyclav 50mg",CEILING($B$8*20/50,0.25)&amp;" tablets",IF(L9="Amoxyclav 250mg",CEILING($B$8*20/250,0.25)&amp;" tablets",IF(L9="Amoxyclav 500mg",CEILING($B$8*20/500,0.25)&amp;" tablets",IF(L9="Doxycycline 50mg",CEILING($B$8*10/50,0.25)&amp;" tablets",IF(L9="Doxycycline 100mg",CEILING($B$8*10/100,0.25)&amp;" tablets",IF(L9="Famvir 125mg",CEILING($B$8*90/125,0.25)&amp;" tablets",IF(L9="Famvir 250mg",CEILING($B$8*90/250,0.25)&amp;" tablets",IF(L9="Meloxicam 1mg (dog tablet)",CEILING($B$8*0.1/1,0.25)&amp;" tablets",IF(L9="Meloxicam 2.5mg (dog tablet)",CEILING($B$8*0.1/2.5,0.25)&amp;" tablets",IF(L9="Clavulox drops (62.5mg/mL)",ROUND($B$8*20/62.5,2)&amp;"mL",IF(L9="Paracetamol 500mg (DOGS ONLY)",CEILING($B$8*15/500,0.25)&amp;" tablets",IF(L9="Doxybrom",ROUND($B$8*0.05,2)&amp;"mL",IF(L9="Panacur",ROUND($B$8/2,2)&amp;"mL",IF(L9="Famvir 250mg/mL solution",ROUND($B$8*90/250,2)&amp;"mL",IF(L9="Mirtazapine 1.88mg (transdermal)","1.88mg",IF(L9="Buprenorphine",ROUND($B$8*0.02/0.3,2)&amp;"mL",IF(L9="Doxycycline paste",CEILING($B$8*10/25,0.5)&amp;" notches",IF(L9="Meloxicam (cat, liquid)",ROUND($B$8*0.1,2)&amp;"mL",IF(L9="Meloxicam (dog, liquid)",ROUND($B$8*0.1/5,2)&amp;"mL",""))))))))))))))))))))</f>
         <v/>
       </c>
       <c r="M12" s="11" t="n"/>
       <c r="N12" s="12" t="n"/>
-      <c r="O12" s="17">
+      <c r="O12" s="69">
         <f>"Dose: "&amp;IF(OR($B$8="",NOT(ISNUMBER($B$8))),"",IF(O9="Amoxyclav 50mg",CEILING($B$8*20/50,0.25)&amp;" tablets",IF(O9="Amoxyclav 250mg",CEILING($B$8*20/250,0.25)&amp;" tablets",IF(O9="Amoxyclav 500mg",CEILING($B$8*20/500,0.25)&amp;" tablets",IF(O9="Doxycycline 50mg",CEILING($B$8*10/50,0.25)&amp;" tablets",IF(O9="Doxycycline 100mg",CEILING($B$8*10/100,0.25)&amp;" tablets",IF(O9="Famvir 125mg",CEILING($B$8*90/125,0.25)&amp;" tablets",IF(O9="Famvir 250mg",CEILING($B$8*90/250,0.25)&amp;" tablets",IF(O9="Meloxicam 1mg (dog tablet)",CEILING($B$8*0.1/1,0.25)&amp;" tablets",IF(O9="Meloxicam 2.5mg (dog tablet)",CEILING($B$8*0.1/2.5,0.25)&amp;" tablets",IF(O9="Clavulox drops (62.5mg/mL)",ROUND($B$8*20/62.5,2)&amp;"mL",IF(O9="Paracetamol 500mg (DOGS ONLY)",CEILING($B$8*15/500,0.25)&amp;" tablets",IF(O9="Doxybrom",ROUND($B$8*0.05,2)&amp;"mL",IF(O9="Panacur",ROUND($B$8/2,2)&amp;"mL",IF(O9="Famvir 250mg/mL solution",ROUND($B$8*90/250,2)&amp;"mL",IF(O9="Mirtazapine 1.88mg (transdermal)","1.88mg",IF(O9="Buprenorphine",ROUND($B$8*0.02/0.3,2)&amp;"mL",IF(O9="Doxycycline paste",CEILING($B$8*10/25,0.5)&amp;" notches",IF(O9="Meloxicam (cat, liquid)",ROUND($B$8*0.1,2)&amp;"mL",IF(O9="Meloxicam (dog, liquid)",ROUND($B$8*0.1/5,2)&amp;"mL",""))))))))))))))))))))</f>
         <v/>
       </c>
@@ -1277,31 +1295,31 @@
       </c>
     </row>
     <row r="13" ht="14" customHeight="1">
-      <c r="C13" s="17">
+      <c r="C13" s="69">
         <f>IF(OR(C9="Amoxyclav 50mg",C9="Amoxyclav 250mg",C9="Amoxyclav 500mg",C9="Clavulox drops (62.5mg/mL)"),"Freq: BID",IF(OR(C9="Doxycycline 50mg",C9="Doxycycline 100mg",C9="Doxycycline paste"),"Freq: SID",IF(ISNUMBER(SEARCH("Meloxicam",C9)),"Freq: SID",IF(C9="Paracetamol 500mg (DOGS ONLY)","Freq: BID",IF(C9="Chlorsig","Freq: BID",IF(OR(C9="Famvir 125mg",C9="Famvir 250mg",C9="Famvir 250mg/mL solution"),"Freq: BID",IF(C9="Doxybrom","Freq: BID",IF(C9="Panacur","Freq: SID",IF(C9="Mirtazapine 1.88mg (transdermal)","Freq: SID",IF(C9="Buprenorphine","Freq: BID","Freq: "))))))))))</f>
         <v/>
       </c>
       <c r="D13" s="11" t="n"/>
       <c r="E13" s="12" t="n"/>
-      <c r="F13" s="17">
+      <c r="F13" s="69">
         <f>IF(OR(F9="Amoxyclav 50mg",F9="Amoxyclav 250mg",F9="Amoxyclav 500mg",F9="Clavulox drops (62.5mg/mL)"),"Freq: BID",IF(OR(F9="Doxycycline 50mg",F9="Doxycycline 100mg",F9="Doxycycline paste"),"Freq: SID",IF(ISNUMBER(SEARCH("Meloxicam",F9)),"Freq: SID",IF(F9="Paracetamol 500mg (DOGS ONLY)","Freq: BID",IF(F9="Chlorsig","Freq: BID",IF(OR(F9="Famvir 125mg",F9="Famvir 250mg",F9="Famvir 250mg/mL solution"),"Freq: BID",IF(F9="Doxybrom","Freq: BID",IF(F9="Panacur","Freq: SID",IF(F9="Mirtazapine 1.88mg (transdermal)","Freq: SID",IF(F9="Buprenorphine","Freq: BID","Freq: "))))))))))</f>
         <v/>
       </c>
       <c r="G13" s="11" t="n"/>
       <c r="H13" s="12" t="n"/>
-      <c r="I13" s="17">
+      <c r="I13" s="69">
         <f>IF(OR(I9="Amoxyclav 50mg",I9="Amoxyclav 250mg",I9="Amoxyclav 500mg",I9="Clavulox drops (62.5mg/mL)"),"Freq: BID",IF(OR(I9="Doxycycline 50mg",I9="Doxycycline 100mg",I9="Doxycycline paste"),"Freq: SID",IF(ISNUMBER(SEARCH("Meloxicam",I9)),"Freq: SID",IF(I9="Paracetamol 500mg (DOGS ONLY)","Freq: BID",IF(I9="Chlorsig","Freq: BID",IF(OR(I9="Famvir 125mg",I9="Famvir 250mg",I9="Famvir 250mg/mL solution"),"Freq: BID",IF(I9="Doxybrom","Freq: BID",IF(I9="Panacur","Freq: SID",IF(I9="Mirtazapine 1.88mg (transdermal)","Freq: SID",IF(I9="Buprenorphine","Freq: BID","Freq: "))))))))))</f>
         <v/>
       </c>
       <c r="J13" s="11" t="n"/>
       <c r="K13" s="12" t="n"/>
-      <c r="L13" s="17">
+      <c r="L13" s="69">
         <f>IF(OR(L9="Amoxyclav 50mg",L9="Amoxyclav 250mg",L9="Amoxyclav 500mg",L9="Clavulox drops (62.5mg/mL)"),"Freq: BID",IF(OR(L9="Doxycycline 50mg",L9="Doxycycline 100mg",L9="Doxycycline paste"),"Freq: SID",IF(ISNUMBER(SEARCH("Meloxicam",L9)),"Freq: SID",IF(L9="Paracetamol 500mg (DOGS ONLY)","Freq: BID",IF(L9="Chlorsig","Freq: BID",IF(OR(L9="Famvir 125mg",L9="Famvir 250mg",L9="Famvir 250mg/mL solution"),"Freq: BID",IF(L9="Doxybrom","Freq: BID",IF(L9="Panacur","Freq: SID",IF(L9="Mirtazapine 1.88mg (transdermal)","Freq: SID",IF(L9="Buprenorphine","Freq: BID","Freq: "))))))))))</f>
         <v/>
       </c>
       <c r="M13" s="11" t="n"/>
       <c r="N13" s="12" t="n"/>
-      <c r="O13" s="17">
+      <c r="O13" s="69">
         <f>IF(OR(O9="Amoxyclav 50mg",O9="Amoxyclav 250mg",O9="Amoxyclav 500mg",O9="Clavulox drops (62.5mg/mL)"),"Freq: BID",IF(OR(O9="Doxycycline 50mg",O9="Doxycycline 100mg",O9="Doxycycline paste"),"Freq: SID",IF(ISNUMBER(SEARCH("Meloxicam",O9)),"Freq: SID",IF(O9="Paracetamol 500mg (DOGS ONLY)","Freq: BID",IF(O9="Chlorsig","Freq: BID",IF(OR(O9="Famvir 125mg",O9="Famvir 250mg",O9="Famvir 250mg/mL solution"),"Freq: BID",IF(O9="Doxybrom","Freq: BID",IF(O9="Panacur","Freq: SID",IF(O9="Mirtazapine 1.88mg (transdermal)","Freq: SID",IF(O9="Buprenorphine","Freq: BID","Freq: "))))))))))</f>
         <v/>
       </c>
@@ -1314,31 +1332,31 @@
       </c>
     </row>
     <row r="14" ht="14" customHeight="1">
-      <c r="C14" s="18">
+      <c r="C14" s="70">
         <f>IF(C9="Chlorsig","Route: Ophthalmic (eye)",IF(C9="Buprenorphine","Route: Transmucosal",IF(C9="Mirtazapine 1.88mg (transdermal)","Route: Transdermal","Route: PO")))</f>
         <v/>
       </c>
       <c r="D14" s="19" t="n"/>
       <c r="E14" s="20" t="n"/>
-      <c r="F14" s="18">
+      <c r="F14" s="70">
         <f>IF(F9="Chlorsig","Route: Ophthalmic (eye)",IF(F9="Buprenorphine","Route: Transmucosal",IF(F9="Mirtazapine 1.88mg (transdermal)","Route: Transdermal","Route: PO")))</f>
         <v/>
       </c>
       <c r="G14" s="19" t="n"/>
       <c r="H14" s="20" t="n"/>
-      <c r="I14" s="18">
+      <c r="I14" s="70">
         <f>IF(I9="Chlorsig","Route: Ophthalmic (eye)",IF(I9="Buprenorphine","Route: Transmucosal",IF(I9="Mirtazapine 1.88mg (transdermal)","Route: Transdermal","Route: PO")))</f>
         <v/>
       </c>
       <c r="J14" s="19" t="n"/>
       <c r="K14" s="20" t="n"/>
-      <c r="L14" s="18">
+      <c r="L14" s="70">
         <f>IF(L9="Chlorsig","Route: Ophthalmic (eye)",IF(L9="Buprenorphine","Route: Transmucosal",IF(L9="Mirtazapine 1.88mg (transdermal)","Route: Transdermal","Route: PO")))</f>
         <v/>
       </c>
       <c r="M14" s="19" t="n"/>
       <c r="N14" s="20" t="n"/>
-      <c r="O14" s="18">
+      <c r="O14" s="70">
         <f>IF(O9="Chlorsig","Route: Ophthalmic (eye)",IF(O9="Buprenorphine","Route: Transmucosal",IF(O9="Mirtazapine 1.88mg (transdermal)","Route: Transdermal","Route: PO")))</f>
         <v/>
       </c>

</xml_diff>